<commit_message>
Rapport du 10 Juin 2026
</commit_message>
<xml_diff>
--- a/Donnees_Promoteurs.xlsx
+++ b/Donnees_Promoteurs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2463BBAB-D7D3-4559-9E45-D05724FC9F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2DCD291-834A-47F7-9D2A-584E4EC37E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7737" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7737" uniqueCount="126">
   <si>
     <t>Date</t>
   </si>
@@ -398,12 +398,6 @@
   </si>
   <si>
     <t>Fallou SOLY1</t>
-  </si>
-  <si>
-    <t>Fallou SOLY2</t>
-  </si>
-  <si>
-    <t>Fallou SOLY3</t>
   </si>
 </sst>
 </file>
@@ -3299,7 +3293,7 @@
         <v>19</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>126</v>
+        <v>79</v>
       </c>
       <c r="H62" s="1"/>
       <c r="I62" s="1" t="s">
@@ -3341,7 +3335,7 @@
         <v>19</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>127</v>
+        <v>79</v>
       </c>
       <c r="H63" s="1"/>
       <c r="I63" s="1" t="s">

</xml_diff>

<commit_message>
Rapport du 11 Juin 2026
</commit_message>
<xml_diff>
--- a/Donnees_Promoteurs.xlsx
+++ b/Donnees_Promoteurs.xlsx
@@ -1432,10 +1432,10 @@
         </is>
       </c>
       <c r="J27" s="1" t="n">
-        <v>0.11111111</v>
+        <v>0.22222222</v>
       </c>
       <c r="K27" s="1" t="n">
-        <v>3111.111</v>
+        <v>6222.222</v>
       </c>
       <c r="L27" s="1"/>
       <c r="M27" s="1" t="n">
@@ -4465,7 +4465,7 @@
         <v>0.041666668</v>
       </c>
       <c r="K80" s="1" t="n">
-        <v>1083.3334</v>
+        <v>791.6667</v>
       </c>
       <c r="L80" s="1" t="n">
         <v>2000.0</v>
@@ -4581,7 +4581,7 @@
         <v>0.29166666</v>
       </c>
       <c r="K82" s="1" t="n">
-        <v>7583.3335</v>
+        <v>5541.6665</v>
       </c>
       <c r="L82" s="1" t="n">
         <v>2000.0</v>
@@ -4929,7 +4929,7 @@
         <v>0.5</v>
       </c>
       <c r="K88" s="1" t="n">
-        <v>13000.0</v>
+        <v>9500.0</v>
       </c>
       <c r="L88" s="1" t="n">
         <v>2000.0</v>
@@ -5045,7 +5045,7 @@
         <v>0.041666668</v>
       </c>
       <c r="K90" s="1" t="n">
-        <v>1083.3334</v>
+        <v>791.6667</v>
       </c>
       <c r="L90" s="1" t="n">
         <v>2000.0</v>
@@ -5103,7 +5103,7 @@
         <v>0.041666668</v>
       </c>
       <c r="K91" s="1" t="n">
-        <v>1083.3334</v>
+        <v>791.6667</v>
       </c>
       <c r="L91" s="1" t="n">
         <v>2000.0</v>

</xml_diff>

<commit_message>
Rapport du 13 Juin 2026
</commit_message>
<xml_diff>
--- a/Donnees_Promoteurs.xlsx
+++ b/Donnees_Promoteurs.xlsx
@@ -35312,10 +35312,10 @@
         </is>
       </c>
       <c r="J650" s="1" t="n">
-        <v>59.8</v>
+        <v>35.2</v>
       </c>
       <c r="K650" s="1" t="n">
-        <v>717600.0</v>
+        <v>422400.0</v>
       </c>
       <c r="L650" s="1"/>
       <c r="M650" s="1"/>
@@ -35987,7 +35987,7 @@
         <v>10.0</v>
       </c>
       <c r="K664" s="1" t="n">
-        <v>260000.0</v>
+        <v>190000.0</v>
       </c>
       <c r="L664" s="1"/>
       <c r="M664" s="1"/>

</xml_diff>

<commit_message>
Rapport du 19 Juiellet 2026
</commit_message>
<xml_diff>
--- a/Donnees_Promoteurs.xlsx
+++ b/Donnees_Promoteurs.xlsx
@@ -70,7 +70,7 @@
     <col min="2" max="2" width="26.43359375" customWidth="true"/>
     <col min="3" max="3" width="8.57421875" customWidth="true"/>
     <col min="4" max="4" width="15.296875" customWidth="true"/>
-    <col min="5" max="5" width="12.61328125" customWidth="true"/>
+    <col min="5" max="5" width="16.5234375" customWidth="true"/>
     <col min="6" max="6" width="8.6953125" customWidth="true"/>
     <col min="7" max="7" width="26.671875" customWidth="true"/>
     <col min="8" max="8" width="9.55078125" customWidth="true"/>
@@ -2034,6 +2034,556 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1" t="inlineStr">
+        <is>
+          <t>Cafe au Lait 3-en-1</t>
+        </is>
+      </c>
+      <c r="J32" s="1" t="n">
+        <v>99.0</v>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>445500.0</v>
+      </c>
+      <c r="L32" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M32" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1" t="n">
+        <v>31.0</v>
+      </c>
+      <c r="P32" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q32" s="1"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1" t="inlineStr">
+        <is>
+          <t>Chocolat 3-en-1 30x120 pcs</t>
+        </is>
+      </c>
+      <c r="J33" s="1" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>1100000.0</v>
+      </c>
+      <c r="L33" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M33" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1" t="n">
+        <v>32.0</v>
+      </c>
+      <c r="P33" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q33" s="1"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 200gx10</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="n">
+        <v>134.0</v>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>804000.0</v>
+      </c>
+      <c r="L34" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M34" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1" t="n">
+        <v>33.0</v>
+      </c>
+      <c r="P34" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q34" s="1"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J35" s="1" t="n">
+        <v>16.0</v>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>176000.0</v>
+      </c>
+      <c r="L35" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M35" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1" t="n">
+        <v>34.0</v>
+      </c>
+      <c r="P35" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q35" s="1"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1" t="inlineStr">
+        <is>
+          <t>Jus Lido</t>
+        </is>
+      </c>
+      <c r="J36" s="1" t="n">
+        <v>200.0</v>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>2200000.0</v>
+      </c>
+      <c r="L36" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M36" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1" t="n">
+        <v>35.0</v>
+      </c>
+      <c r="P36" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q36" s="1"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Junior BLE cereal 230g x 12 sachet</t>
+        </is>
+      </c>
+      <c r="J37" s="1" t="n">
+        <v>24.416666</v>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>219750.0</v>
+      </c>
+      <c r="L37" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M37" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1" t="n">
+        <v>36.0</v>
+      </c>
+      <c r="P37" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q37" s="1"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Junior BLE cereal 50g x 10 x 8 sachet</t>
+        </is>
+      </c>
+      <c r="J38" s="1" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>375000.0</v>
+      </c>
+      <c r="L38" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M38" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1" t="n">
+        <v>37.0</v>
+      </c>
+      <c r="P38" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q38" s="1"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Junior mais cereal 230g x 12 sachet</t>
+        </is>
+      </c>
+      <c r="J39" s="1" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>225000.0</v>
+      </c>
+      <c r="L39" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M39" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1" t="n">
+        <v>38.0</v>
+      </c>
+      <c r="P39" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q39" s="1"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Junior mais cereal 50g x 10 x 8 sachet</t>
+        </is>
+      </c>
+      <c r="J40" s="1" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>375000.0</v>
+      </c>
+      <c r="L40" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M40" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N40" s="1"/>
+      <c r="O40" s="1" t="n">
+        <v>39.0</v>
+      </c>
+      <c r="P40" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q40" s="1"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Thé 7g</t>
+        </is>
+      </c>
+      <c r="J41" s="1" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>1150000.0</v>
+      </c>
+      <c r="L41" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M41" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N41" s="1"/>
+      <c r="O41" s="1" t="n">
+        <v>40.0</v>
+      </c>
+      <c r="P41" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q41" s="1"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Rapport du 19 juillet 2026
</commit_message>
<xml_diff>
--- a/Donnees_Promoteurs.xlsx
+++ b/Donnees_Promoteurs.xlsx
@@ -174,7 +174,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0.0</v>
@@ -191,7 +191,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -199,39 +199,47 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G2" s="1"/>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Saliou KONE</t>
+        </is>
+      </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>Kamlac évaporé 48x160g</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J2" s="1" t="n">
-        <v>600.0</v>
+        <v>2.0</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>6300000.0</v>
+        <v>22000.0</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.0</v>
+        <v>5000.0</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>0.0</v>
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="1" t="n">
-        <v>1.0</v>
+        <v>42.0</v>
       </c>
       <c r="P2" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q2" s="1"/>
+      <c r="Q2" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>0.0</v>
@@ -248,7 +256,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
@@ -256,18 +264,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G3" s="1"/>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Saliou KONE</t>
+        </is>
+      </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="inlineStr">
         <is>
-          <t>Jus Lido</t>
+          <t>Cowmilk 200gx10</t>
         </is>
       </c>
       <c r="J3" s="1" t="n">
-        <v>200.0</v>
+        <v>1.0</v>
       </c>
       <c r="K3" s="1" t="n">
-        <v>2200000.0</v>
+        <v>6000.0</v>
       </c>
       <c r="L3" s="1" t="n">
         <v>0.0</v>
@@ -277,18 +289,22 @@
       </c>
       <c r="N3" s="1"/>
       <c r="O3" s="1" t="n">
-        <v>2.0</v>
+        <v>43.0</v>
       </c>
       <c r="P3" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q3" s="1"/>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>0.0</v>
@@ -305,7 +321,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -313,7 +329,11 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G4" s="1"/>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Saliou KONE</t>
+        </is>
+      </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1" t="inlineStr">
         <is>
@@ -321,10 +341,10 @@
         </is>
       </c>
       <c r="J4" s="1" t="n">
-        <v>100.0</v>
+        <v>1.0</v>
       </c>
       <c r="K4" s="1" t="n">
-        <v>450000.0</v>
+        <v>4500.0</v>
       </c>
       <c r="L4" s="1" t="n">
         <v>0.0</v>
@@ -334,18 +354,22 @@
       </c>
       <c r="N4" s="1"/>
       <c r="O4" s="1" t="n">
-        <v>3.0</v>
+        <v>44.0</v>
       </c>
       <c r="P4" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q4" s="1"/>
+      <c r="Q4" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.0</v>
@@ -362,7 +386,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -370,18 +394,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G5" s="1"/>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>Adama DABO</t>
+        </is>
+      </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1" t="inlineStr">
         <is>
-          <t>Chocolat 3-en-1 30x120 pcs</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J5" s="1" t="n">
-        <v>100.0</v>
+        <v>2.0</v>
       </c>
       <c r="K5" s="1" t="n">
-        <v>1100000.0</v>
+        <v>22000.0</v>
       </c>
       <c r="L5" s="1" t="n">
         <v>0.0</v>
@@ -391,18 +419,22 @@
       </c>
       <c r="N5" s="1"/>
       <c r="O5" s="1" t="n">
-        <v>4.0</v>
+        <v>45.0</v>
       </c>
       <c r="P5" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q5" s="1"/>
+      <c r="Q5" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.0</v>
@@ -419,7 +451,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -427,18 +459,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G6" s="1"/>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Adama DABO</t>
+        </is>
+      </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Thé 7g</t>
+          <t>Cowmilk 200gx10</t>
         </is>
       </c>
       <c r="J6" s="1" t="n">
-        <v>100.0</v>
+        <v>2.0</v>
       </c>
       <c r="K6" s="1" t="n">
-        <v>1150000.0</v>
+        <v>12000.0</v>
       </c>
       <c r="L6" s="1" t="n">
         <v>0.0</v>
@@ -448,18 +484,22 @@
       </c>
       <c r="N6" s="1"/>
       <c r="O6" s="1" t="n">
-        <v>5.0</v>
+        <v>46.0</v>
       </c>
       <c r="P6" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q6" s="1"/>
+      <c r="Q6" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.0</v>
@@ -476,7 +516,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
@@ -484,18 +524,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G7" s="1"/>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>Adama DABO</t>
+        </is>
+      </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Kamlac évaporé 48x160g</t>
         </is>
       </c>
       <c r="J7" s="1" t="n">
-        <v>100.0</v>
+        <v>3.0</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>1100000.0</v>
+        <v>31500.0</v>
       </c>
       <c r="L7" s="1" t="n">
         <v>0.0</v>
@@ -505,18 +549,22 @@
       </c>
       <c r="N7" s="1"/>
       <c r="O7" s="1" t="n">
-        <v>6.0</v>
+        <v>47.0</v>
       </c>
       <c r="P7" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q7" s="1"/>
+      <c r="Q7" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.0</v>
@@ -533,7 +581,7 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
@@ -541,18 +589,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G8" s="1"/>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Adama DABO</t>
+        </is>
+      </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 200gx10</t>
+          <t>Kamlac Junior BLE cereal 230g x 12 sachet</t>
         </is>
       </c>
       <c r="J8" s="1" t="n">
-        <v>140.0</v>
+        <v>1.0</v>
       </c>
       <c r="K8" s="1" t="n">
-        <v>840000.0</v>
+        <v>9000.0</v>
       </c>
       <c r="L8" s="1" t="n">
         <v>0.0</v>
@@ -562,18 +614,22 @@
       </c>
       <c r="N8" s="1"/>
       <c r="O8" s="1" t="n">
-        <v>7.0</v>
+        <v>48.0</v>
       </c>
       <c r="P8" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q8" s="1"/>
+      <c r="Q8" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.0</v>
@@ -590,7 +646,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
@@ -598,18 +654,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Adama DABO</t>
+        </is>
+      </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Junior BLE cereal 50g x 10 x 8 sachet</t>
+          <t>Kamlac Thé 7g</t>
         </is>
       </c>
       <c r="J9" s="1" t="n">
-        <v>25.0</v>
+        <v>0.25</v>
       </c>
       <c r="K9" s="1" t="n">
-        <v>375000.0</v>
+        <v>2875.0</v>
       </c>
       <c r="L9" s="1" t="n">
         <v>0.0</v>
@@ -619,18 +679,22 @@
       </c>
       <c r="N9" s="1"/>
       <c r="O9" s="1" t="n">
-        <v>8.0</v>
+        <v>49.0</v>
       </c>
       <c r="P9" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q9" s="1"/>
+      <c r="Q9" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.0</v>
@@ -647,7 +711,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
@@ -655,18 +719,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G10" s="1"/>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Saly THIOUNE (T2)</t>
+        </is>
+      </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Junior mais cereal 50g x 10 x 8 sachet</t>
+          <t>Kamlac évaporé 48x160g</t>
         </is>
       </c>
       <c r="J10" s="1" t="n">
-        <v>25.0</v>
+        <v>2.0</v>
       </c>
       <c r="K10" s="1" t="n">
-        <v>375000.0</v>
+        <v>21000.0</v>
       </c>
       <c r="L10" s="1" t="n">
         <v>0.0</v>
@@ -676,18 +744,22 @@
       </c>
       <c r="N10" s="1"/>
       <c r="O10" s="1" t="n">
-        <v>9.0</v>
+        <v>50.0</v>
       </c>
       <c r="P10" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q10" s="1"/>
+      <c r="Q10" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.0</v>
@@ -704,7 +776,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
@@ -712,18 +784,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G11" s="1"/>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Sokhna (T2)</t>
+        </is>
+      </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Junior mais cereal 230g x 12 sachet</t>
+          <t>Kamlac évaporé 48x160g</t>
         </is>
       </c>
       <c r="J11" s="1" t="n">
-        <v>25.0</v>
+        <v>1.0</v>
       </c>
       <c r="K11" s="1" t="n">
-        <v>225000.0</v>
+        <v>10500.0</v>
       </c>
       <c r="L11" s="1" t="n">
         <v>0.0</v>
@@ -733,18 +809,22 @@
       </c>
       <c r="N11" s="1"/>
       <c r="O11" s="1" t="n">
-        <v>10.0</v>
+        <v>51.0</v>
       </c>
       <c r="P11" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q11" s="1"/>
+      <c r="Q11" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.0</v>
@@ -761,7 +841,7 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Stock Lundi</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
@@ -769,18 +849,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G12" s="1"/>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>Sokhna (T2)</t>
+        </is>
+      </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Junior BLE cereal 230g x 12 sachet</t>
+          <t>Cowmilk 200gx10</t>
         </is>
       </c>
       <c r="J12" s="1" t="n">
-        <v>25.0</v>
+        <v>0.5</v>
       </c>
       <c r="K12" s="1" t="n">
-        <v>225000.0</v>
+        <v>3000.0</v>
       </c>
       <c r="L12" s="1" t="n">
         <v>0.0</v>
@@ -790,18 +874,22 @@
       </c>
       <c r="N12" s="1"/>
       <c r="O12" s="1" t="n">
-        <v>11.0</v>
+        <v>52.0</v>
       </c>
       <c r="P12" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q12" s="1"/>
+      <c r="Q12" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.0</v>
@@ -828,7 +916,7 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>Jackline DIEDHIOU (T3)</t>
+          <t>Sokhna (T2)</t>
         </is>
       </c>
       <c r="H13" s="1"/>
@@ -838,20 +926,20 @@
         </is>
       </c>
       <c r="J13" s="1" t="n">
-        <v>0.5833333</v>
+        <v>1.0</v>
       </c>
       <c r="K13" s="1" t="n">
-        <v>5250.0</v>
+        <v>9000.0</v>
       </c>
       <c r="L13" s="1" t="n">
-        <v>10000.0</v>
+        <v>0.0</v>
       </c>
       <c r="M13" s="1" t="n">
         <v>0.0</v>
       </c>
       <c r="N13" s="1"/>
       <c r="O13" s="1" t="n">
-        <v>12.0</v>
+        <v>53.0</v>
       </c>
       <c r="P13" s="1" t="inlineStr">
         <is>
@@ -866,7 +954,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.0</v>
@@ -893,20 +981,20 @@
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>Jackline DIEDHIOU (T3)</t>
+          <t>Ndeye Fatou GUEYE (T3)</t>
         </is>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Cowmilk 200gx10</t>
         </is>
       </c>
       <c r="J14" s="1" t="n">
-        <v>6.0</v>
+        <v>0.5</v>
       </c>
       <c r="K14" s="1" t="n">
-        <v>66000.0</v>
+        <v>3000.0</v>
       </c>
       <c r="L14" s="1" t="n">
         <v>0.0</v>
@@ -916,7 +1004,7 @@
       </c>
       <c r="N14" s="1"/>
       <c r="O14" s="1" t="n">
-        <v>13.0</v>
+        <v>54.0</v>
       </c>
       <c r="P14" s="1" t="inlineStr">
         <is>
@@ -931,7 +1019,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.0</v>
@@ -958,20 +1046,20 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>Ndeye Fatou GUEYE (T3)</t>
+          <t>Jackline DIEDHIOU (T3)</t>
         </is>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Cowmilk 200gx10</t>
         </is>
       </c>
       <c r="J15" s="1" t="n">
-        <v>6.0</v>
+        <v>0.5</v>
       </c>
       <c r="K15" s="1" t="n">
-        <v>66000.0</v>
+        <v>3000.0</v>
       </c>
       <c r="L15" s="1" t="n">
         <v>0.0</v>
@@ -981,7 +1069,7 @@
       </c>
       <c r="N15" s="1"/>
       <c r="O15" s="1" t="n">
-        <v>14.0</v>
+        <v>55.0</v>
       </c>
       <c r="P15" s="1" t="inlineStr">
         <is>
@@ -996,7 +1084,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.0</v>
@@ -1023,7 +1111,7 @@
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>Saliou KONE</t>
+          <t>Fama DIOUF</t>
         </is>
       </c>
       <c r="H16" s="1"/>
@@ -1033,10 +1121,10 @@
         </is>
       </c>
       <c r="J16" s="1" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="K16" s="1" t="n">
-        <v>66000.0</v>
+        <v>55000.0</v>
       </c>
       <c r="L16" s="1" t="n">
         <v>0.0</v>
@@ -1046,7 +1134,7 @@
       </c>
       <c r="N16" s="1"/>
       <c r="O16" s="1" t="n">
-        <v>15.0</v>
+        <v>56.0</v>
       </c>
       <c r="P16" s="1" t="inlineStr">
         <is>
@@ -1061,7 +1149,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.0</v>
@@ -1088,20 +1176,20 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>Saliou KONE</t>
+          <t>Mariama KANE</t>
         </is>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="inlineStr">
         <is>
-          <t>Kamlac évaporé 48x160g</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J17" s="1" t="n">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="K17" s="1" t="n">
-        <v>10500.0</v>
+        <v>55000.0</v>
       </c>
       <c r="L17" s="1" t="n">
         <v>0.0</v>
@@ -1111,7 +1199,7 @@
       </c>
       <c r="N17" s="1"/>
       <c r="O17" s="1" t="n">
-        <v>16.0</v>
+        <v>57.0</v>
       </c>
       <c r="P17" s="1" t="inlineStr">
         <is>
@@ -1126,7 +1214,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.0</v>
@@ -1153,20 +1241,20 @@
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>Saliou KONE</t>
+          <t>Fallou SOLY (T2)</t>
         </is>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 200gx10</t>
+          <t>Kamlac Thé 7g</t>
         </is>
       </c>
       <c r="J18" s="1" t="n">
-        <v>2.0</v>
+        <v>0.25</v>
       </c>
       <c r="K18" s="1" t="n">
-        <v>12000.0</v>
+        <v>2875.0</v>
       </c>
       <c r="L18" s="1" t="n">
         <v>0.0</v>
@@ -1176,7 +1264,7 @@
       </c>
       <c r="N18" s="1"/>
       <c r="O18" s="1" t="n">
-        <v>17.0</v>
+        <v>58.0</v>
       </c>
       <c r="P18" s="1" t="inlineStr">
         <is>
@@ -1191,7 +1279,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.0</v>
@@ -1218,20 +1306,20 @@
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>Adama DABO</t>
+          <t>Mariama BA</t>
         </is>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Kamlac Thé 7g</t>
         </is>
       </c>
       <c r="J19" s="1" t="n">
-        <v>7.0</v>
+        <v>0.25</v>
       </c>
       <c r="K19" s="1" t="n">
-        <v>77000.0</v>
+        <v>2875.0</v>
       </c>
       <c r="L19" s="1" t="n">
         <v>0.0</v>
@@ -1241,7 +1329,7 @@
       </c>
       <c r="N19" s="1"/>
       <c r="O19" s="1" t="n">
-        <v>18.0</v>
+        <v>59.0</v>
       </c>
       <c r="P19" s="1" t="inlineStr">
         <is>
@@ -1256,7 +1344,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.0</v>
@@ -1283,20 +1371,20 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>Adama DABO</t>
+          <t>Coumba Touré (T2)</t>
         </is>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 200gx10</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J20" s="1" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="K20" s="1" t="n">
-        <v>12000.0</v>
+        <v>11000.0</v>
       </c>
       <c r="L20" s="1" t="n">
         <v>0.0</v>
@@ -1306,7 +1394,7 @@
       </c>
       <c r="N20" s="1"/>
       <c r="O20" s="1" t="n">
-        <v>19.0</v>
+        <v>60.0</v>
       </c>
       <c r="P20" s="1" t="inlineStr">
         <is>
@@ -1321,7 +1409,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.0</v>
@@ -1348,20 +1436,20 @@
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>Saly THIOUNE (T2)</t>
+          <t>Coumba Touré (T2)</t>
         </is>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Kamlac évaporé 48x160g</t>
         </is>
       </c>
       <c r="J21" s="1" t="n">
         <v>1.0</v>
       </c>
       <c r="K21" s="1" t="n">
-        <v>11000.0</v>
+        <v>10500.0</v>
       </c>
       <c r="L21" s="1" t="n">
         <v>0.0</v>
@@ -1371,7 +1459,7 @@
       </c>
       <c r="N21" s="1"/>
       <c r="O21" s="1" t="n">
-        <v>20.0</v>
+        <v>61.0</v>
       </c>
       <c r="P21" s="1" t="inlineStr">
         <is>
@@ -1386,7 +1474,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.0</v>
@@ -1413,21 +1501,19 @@
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>Sokhna (T2)</t>
+          <t>Coumba Touré (T2)</t>
         </is>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Kamlac Thé 7g</t>
         </is>
       </c>
       <c r="J22" s="1" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="K22" s="1" t="n">
-        <v>22000.0</v>
-      </c>
+        <v>0.45833334</v>
+      </c>
+      <c r="K22" s="1"/>
       <c r="L22" s="1" t="n">
         <v>0.0</v>
       </c>
@@ -1436,7 +1522,7 @@
       </c>
       <c r="N22" s="1"/>
       <c r="O22" s="1" t="n">
-        <v>21.0</v>
+        <v>62.0</v>
       </c>
       <c r="P22" s="1" t="inlineStr">
         <is>
@@ -1451,7 +1537,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.0</v>
@@ -1478,20 +1564,20 @@
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>Sokhna (T2)</t>
+          <t>Nogueye THIAME (T2)</t>
         </is>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 200gx10</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J23" s="1" t="n">
         <v>1.0</v>
       </c>
       <c r="K23" s="1" t="n">
-        <v>6000.0</v>
+        <v>11000.0</v>
       </c>
       <c r="L23" s="1" t="n">
         <v>0.0</v>
@@ -1501,7 +1587,7 @@
       </c>
       <c r="N23" s="1"/>
       <c r="O23" s="1" t="n">
-        <v>22.0</v>
+        <v>63.0</v>
       </c>
       <c r="P23" s="1" t="inlineStr">
         <is>
@@ -1516,7 +1602,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46221.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>0.0</v>
@@ -1549,14 +1635,14 @@
       <c r="H24" s="1"/>
       <c r="I24" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Cafe au Lait 3-en-1</t>
         </is>
       </c>
       <c r="J24" s="1" t="n">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
       <c r="K24" s="1" t="n">
-        <v>110000.0</v>
+        <v>4500.0</v>
       </c>
       <c r="L24" s="1" t="n">
         <v>0.0</v>
@@ -1566,7 +1652,7 @@
       </c>
       <c r="N24" s="1"/>
       <c r="O24" s="1" t="n">
-        <v>23.0</v>
+        <v>64.0</v>
       </c>
       <c r="P24" s="1" t="inlineStr">
         <is>
@@ -1598,7 +1684,7 @@
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>Vente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
@@ -1606,22 +1692,18 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G25" s="1" t="inlineStr">
-        <is>
-          <t>Coumba Touré (T2)</t>
-        </is>
-      </c>
+      <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Kamlac évaporé 48x160g</t>
         </is>
       </c>
       <c r="J25" s="1" t="n">
-        <v>11.0</v>
+        <v>600.0</v>
       </c>
       <c r="K25" s="1" t="n">
-        <v>121000.0</v>
+        <v>6300000.0</v>
       </c>
       <c r="L25" s="1" t="n">
         <v>0.0</v>
@@ -1631,18 +1713,14 @@
       </c>
       <c r="N25" s="1"/>
       <c r="O25" s="1" t="n">
-        <v>24.0</v>
+        <v>1.0</v>
       </c>
       <c r="P25" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q25" s="1" t="inlineStr">
-        <is>
-          <t>Equipe</t>
-        </is>
-      </c>
+      <c r="Q25" s="1"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1663,7 +1741,7 @@
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>Vente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
@@ -1671,22 +1749,18 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G26" s="1" t="inlineStr">
-        <is>
-          <t>Fama DIOUF</t>
-        </is>
-      </c>
+      <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Jus Lido</t>
         </is>
       </c>
       <c r="J26" s="1" t="n">
-        <v>5.0</v>
+        <v>200.0</v>
       </c>
       <c r="K26" s="1" t="n">
-        <v>55000.0</v>
+        <v>2200000.0</v>
       </c>
       <c r="L26" s="1" t="n">
         <v>0.0</v>
@@ -1696,18 +1770,14 @@
       </c>
       <c r="N26" s="1"/>
       <c r="O26" s="1" t="n">
-        <v>25.0</v>
+        <v>2.0</v>
       </c>
       <c r="P26" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q26" s="1" t="inlineStr">
-        <is>
-          <t>Equipe</t>
-        </is>
-      </c>
+      <c r="Q26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1728,7 +1798,7 @@
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>Vente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
@@ -1736,22 +1806,18 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G27" s="1" t="inlineStr">
-        <is>
-          <t>Mariama KANE</t>
-        </is>
-      </c>
+      <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Cafe au Lait 3-en-1</t>
         </is>
       </c>
       <c r="J27" s="1" t="n">
-        <v>5.0</v>
+        <v>100.0</v>
       </c>
       <c r="K27" s="1" t="n">
-        <v>55000.0</v>
+        <v>450000.0</v>
       </c>
       <c r="L27" s="1" t="n">
         <v>0.0</v>
@@ -1761,18 +1827,14 @@
       </c>
       <c r="N27" s="1"/>
       <c r="O27" s="1" t="n">
-        <v>26.0</v>
+        <v>3.0</v>
       </c>
       <c r="P27" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q27" s="1" t="inlineStr">
-        <is>
-          <t>Equipe</t>
-        </is>
-      </c>
+      <c r="Q27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1793,7 +1855,7 @@
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>Vente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
@@ -1801,22 +1863,18 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G28" s="1" t="inlineStr">
-        <is>
-          <t>Mariama KANE</t>
-        </is>
-      </c>
+      <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 200gx10</t>
+          <t>Chocolat 3-en-1 30x120 pcs</t>
         </is>
       </c>
       <c r="J28" s="1" t="n">
-        <v>1.0</v>
+        <v>100.0</v>
       </c>
       <c r="K28" s="1" t="n">
-        <v>6000.0</v>
+        <v>1100000.0</v>
       </c>
       <c r="L28" s="1" t="n">
         <v>0.0</v>
@@ -1826,18 +1884,14 @@
       </c>
       <c r="N28" s="1"/>
       <c r="O28" s="1" t="n">
-        <v>27.0</v>
+        <v>4.0</v>
       </c>
       <c r="P28" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q28" s="1" t="inlineStr">
-        <is>
-          <t>Equipe</t>
-        </is>
-      </c>
+      <c r="Q28" s="1"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1858,7 +1912,7 @@
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>Vente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
@@ -1866,22 +1920,18 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G29" s="1" t="inlineStr">
-        <is>
-          <t>Fallou SOLY (T2)</t>
-        </is>
-      </c>
+      <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Kamlac Thé 7g</t>
         </is>
       </c>
       <c r="J29" s="1" t="n">
-        <v>15.0</v>
+        <v>100.0</v>
       </c>
       <c r="K29" s="1" t="n">
-        <v>165000.0</v>
+        <v>1150000.0</v>
       </c>
       <c r="L29" s="1" t="n">
         <v>0.0</v>
@@ -1891,18 +1941,14 @@
       </c>
       <c r="N29" s="1"/>
       <c r="O29" s="1" t="n">
-        <v>28.0</v>
+        <v>5.0</v>
       </c>
       <c r="P29" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q29" s="1" t="inlineStr">
-        <is>
-          <t>Equipe</t>
-        </is>
-      </c>
+      <c r="Q29" s="1"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1923,7 +1969,7 @@
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>Vente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
@@ -1931,22 +1977,18 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G30" s="1" t="inlineStr">
-        <is>
-          <t>Fallou SOLY (T2)</t>
-        </is>
-      </c>
+      <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1" t="inlineStr">
         <is>
-          <t>Cafe au Lait 3-en-1</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J30" s="1" t="n">
-        <v>1.0</v>
+        <v>100.0</v>
       </c>
       <c r="K30" s="1" t="n">
-        <v>4500.0</v>
+        <v>1100000.0</v>
       </c>
       <c r="L30" s="1" t="n">
         <v>0.0</v>
@@ -1956,18 +1998,14 @@
       </c>
       <c r="N30" s="1"/>
       <c r="O30" s="1" t="n">
-        <v>29.0</v>
+        <v>6.0</v>
       </c>
       <c r="P30" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q30" s="1" t="inlineStr">
-        <is>
-          <t>Equipe</t>
-        </is>
-      </c>
+      <c r="Q30" s="1"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1988,7 +2026,7 @@
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>Vente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
@@ -1996,22 +2034,18 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G31" s="1" t="inlineStr">
-        <is>
-          <t>Mariama BA</t>
-        </is>
-      </c>
+      <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Cowmilk 200gx10</t>
         </is>
       </c>
       <c r="J31" s="1" t="n">
-        <v>10.0</v>
+        <v>140.0</v>
       </c>
       <c r="K31" s="1" t="n">
-        <v>110000.0</v>
+        <v>840000.0</v>
       </c>
       <c r="L31" s="1" t="n">
         <v>0.0</v>
@@ -2021,18 +2055,14 @@
       </c>
       <c r="N31" s="1"/>
       <c r="O31" s="1" t="n">
-        <v>30.0</v>
+        <v>7.0</v>
       </c>
       <c r="P31" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q31" s="1" t="inlineStr">
-        <is>
-          <t>Equipe</t>
-        </is>
-      </c>
+      <c r="Q31" s="1"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2053,7 +2083,7 @@
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
@@ -2065,14 +2095,14 @@
       <c r="H32" s="1"/>
       <c r="I32" s="1" t="inlineStr">
         <is>
-          <t>Cafe au Lait 3-en-1</t>
+          <t>Kamlac Junior BLE cereal 50g x 10 x 8 sachet</t>
         </is>
       </c>
       <c r="J32" s="1" t="n">
-        <v>99.0</v>
+        <v>25.0</v>
       </c>
       <c r="K32" s="1" t="n">
-        <v>445500.0</v>
+        <v>375000.0</v>
       </c>
       <c r="L32" s="1" t="n">
         <v>0.0</v>
@@ -2082,7 +2112,7 @@
       </c>
       <c r="N32" s="1"/>
       <c r="O32" s="1" t="n">
-        <v>31.0</v>
+        <v>8.0</v>
       </c>
       <c r="P32" s="1" t="inlineStr">
         <is>
@@ -2110,7 +2140,7 @@
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
@@ -2122,14 +2152,14 @@
       <c r="H33" s="1"/>
       <c r="I33" s="1" t="inlineStr">
         <is>
-          <t>Chocolat 3-en-1 30x120 pcs</t>
+          <t>Kamlac Junior mais cereal 50g x 10 x 8 sachet</t>
         </is>
       </c>
       <c r="J33" s="1" t="n">
-        <v>100.0</v>
+        <v>25.0</v>
       </c>
       <c r="K33" s="1" t="n">
-        <v>1100000.0</v>
+        <v>375000.0</v>
       </c>
       <c r="L33" s="1" t="n">
         <v>0.0</v>
@@ -2139,7 +2169,7 @@
       </c>
       <c r="N33" s="1"/>
       <c r="O33" s="1" t="n">
-        <v>32.0</v>
+        <v>9.0</v>
       </c>
       <c r="P33" s="1" t="inlineStr">
         <is>
@@ -2167,7 +2197,7 @@
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
@@ -2179,14 +2209,14 @@
       <c r="H34" s="1"/>
       <c r="I34" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 200gx10</t>
+          <t>Kamlac Junior mais cereal 230g x 12 sachet</t>
         </is>
       </c>
       <c r="J34" s="1" t="n">
-        <v>134.0</v>
+        <v>25.0</v>
       </c>
       <c r="K34" s="1" t="n">
-        <v>804000.0</v>
+        <v>225000.0</v>
       </c>
       <c r="L34" s="1" t="n">
         <v>0.0</v>
@@ -2196,7 +2226,7 @@
       </c>
       <c r="N34" s="1"/>
       <c r="O34" s="1" t="n">
-        <v>33.0</v>
+        <v>10.0</v>
       </c>
       <c r="P34" s="1" t="inlineStr">
         <is>
@@ -2224,7 +2254,7 @@
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Stock Lundi</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
@@ -2236,14 +2266,14 @@
       <c r="H35" s="1"/>
       <c r="I35" s="1" t="inlineStr">
         <is>
-          <t>Cowmilk 5kg</t>
+          <t>Kamlac Junior BLE cereal 230g x 12 sachet</t>
         </is>
       </c>
       <c r="J35" s="1" t="n">
-        <v>16.0</v>
+        <v>25.0</v>
       </c>
       <c r="K35" s="1" t="n">
-        <v>176000.0</v>
+        <v>225000.0</v>
       </c>
       <c r="L35" s="1" t="n">
         <v>0.0</v>
@@ -2253,7 +2283,7 @@
       </c>
       <c r="N35" s="1"/>
       <c r="O35" s="1" t="n">
-        <v>34.0</v>
+        <v>11.0</v>
       </c>
       <c r="P35" s="1" t="inlineStr">
         <is>
@@ -2281,7 +2311,7 @@
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
@@ -2289,35 +2319,43 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G36" s="1"/>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>Jackline DIEDHIOU (T3)</t>
+        </is>
+      </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1" t="inlineStr">
         <is>
-          <t>Jus Lido</t>
+          <t>Kamlac Junior BLE cereal 230g x 12 sachet</t>
         </is>
       </c>
       <c r="J36" s="1" t="n">
-        <v>200.0</v>
+        <v>0.5833333</v>
       </c>
       <c r="K36" s="1" t="n">
-        <v>2200000.0</v>
+        <v>5250.0</v>
       </c>
       <c r="L36" s="1" t="n">
-        <v>0.0</v>
+        <v>10000.0</v>
       </c>
       <c r="M36" s="1" t="n">
         <v>0.0</v>
       </c>
       <c r="N36" s="1"/>
       <c r="O36" s="1" t="n">
-        <v>35.0</v>
+        <v>12.0</v>
       </c>
       <c r="P36" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q36" s="1"/>
+      <c r="Q36" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2338,7 +2376,7 @@
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
@@ -2346,18 +2384,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G37" s="1"/>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>Jackline DIEDHIOU (T3)</t>
+        </is>
+      </c>
       <c r="H37" s="1"/>
       <c r="I37" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Junior BLE cereal 230g x 12 sachet</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J37" s="1" t="n">
-        <v>24.416666</v>
+        <v>6.0</v>
       </c>
       <c r="K37" s="1" t="n">
-        <v>219750.0</v>
+        <v>66000.0</v>
       </c>
       <c r="L37" s="1" t="n">
         <v>0.0</v>
@@ -2367,14 +2409,18 @@
       </c>
       <c r="N37" s="1"/>
       <c r="O37" s="1" t="n">
-        <v>36.0</v>
+        <v>13.0</v>
       </c>
       <c r="P37" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q37" s="1"/>
+      <c r="Q37" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2395,7 +2441,7 @@
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
@@ -2403,18 +2449,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G38" s="1"/>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>Ndeye Fatou GUEYE (T3)</t>
+        </is>
+      </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Junior BLE cereal 50g x 10 x 8 sachet</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J38" s="1" t="n">
-        <v>25.0</v>
+        <v>6.0</v>
       </c>
       <c r="K38" s="1" t="n">
-        <v>375000.0</v>
+        <v>66000.0</v>
       </c>
       <c r="L38" s="1" t="n">
         <v>0.0</v>
@@ -2424,14 +2474,18 @@
       </c>
       <c r="N38" s="1"/>
       <c r="O38" s="1" t="n">
-        <v>37.0</v>
+        <v>14.0</v>
       </c>
       <c r="P38" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q38" s="1"/>
+      <c r="Q38" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2452,7 +2506,7 @@
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
@@ -2460,18 +2514,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G39" s="1"/>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>Saliou KONE</t>
+        </is>
+      </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Junior mais cereal 230g x 12 sachet</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J39" s="1" t="n">
-        <v>25.0</v>
+        <v>6.0</v>
       </c>
       <c r="K39" s="1" t="n">
-        <v>225000.0</v>
+        <v>66000.0</v>
       </c>
       <c r="L39" s="1" t="n">
         <v>0.0</v>
@@ -2481,14 +2539,18 @@
       </c>
       <c r="N39" s="1"/>
       <c r="O39" s="1" t="n">
-        <v>38.0</v>
+        <v>15.0</v>
       </c>
       <c r="P39" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q39" s="1"/>
+      <c r="Q39" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2509,7 +2571,7 @@
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
@@ -2517,18 +2579,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G40" s="1"/>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>Saliou KONE</t>
+        </is>
+      </c>
       <c r="H40" s="1"/>
       <c r="I40" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Junior mais cereal 50g x 10 x 8 sachet</t>
+          <t>Kamlac évaporé 48x160g</t>
         </is>
       </c>
       <c r="J40" s="1" t="n">
-        <v>25.0</v>
+        <v>1.0</v>
       </c>
       <c r="K40" s="1" t="n">
-        <v>375000.0</v>
+        <v>10500.0</v>
       </c>
       <c r="L40" s="1" t="n">
         <v>0.0</v>
@@ -2538,14 +2604,18 @@
       </c>
       <c r="N40" s="1"/>
       <c r="O40" s="1" t="n">
-        <v>39.0</v>
+        <v>16.0</v>
       </c>
       <c r="P40" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q40" s="1"/>
+      <c r="Q40" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2566,7 +2636,7 @@
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
@@ -2574,18 +2644,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G41" s="1"/>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>Saliou KONE</t>
+        </is>
+      </c>
       <c r="H41" s="1"/>
       <c r="I41" s="1" t="inlineStr">
         <is>
-          <t>Kamlac Thé 7g</t>
+          <t>Cowmilk 200gx10</t>
         </is>
       </c>
       <c r="J41" s="1" t="n">
-        <v>100.0</v>
+        <v>2.0</v>
       </c>
       <c r="K41" s="1" t="n">
-        <v>1150000.0</v>
+        <v>12000.0</v>
       </c>
       <c r="L41" s="1" t="n">
         <v>0.0</v>
@@ -2595,14 +2669,18 @@
       </c>
       <c r="N41" s="1"/>
       <c r="O41" s="1" t="n">
-        <v>40.0</v>
+        <v>17.0</v>
       </c>
       <c r="P41" s="1" t="inlineStr">
         <is>
           <t>S29</t>
         </is>
       </c>
-      <c r="Q41" s="1"/>
+      <c r="Q41" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2623,7 +2701,7 @@
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>Stock Descente</t>
+          <t>Vente</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
@@ -2631,18 +2709,22 @@
           <t>TOUBA</t>
         </is>
       </c>
-      <c r="G42" s="1"/>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>Adama DABO</t>
+        </is>
+      </c>
       <c r="H42" s="1"/>
       <c r="I42" s="1" t="inlineStr">
         <is>
-          <t>Kamlac évaporé 48x160g</t>
+          <t>Cowmilk 5kg</t>
         </is>
       </c>
       <c r="J42" s="1" t="n">
-        <v>599.0</v>
+        <v>7.0</v>
       </c>
       <c r="K42" s="1" t="n">
-        <v>6289500.0</v>
+        <v>77000.0</v>
       </c>
       <c r="L42" s="1" t="n">
         <v>0.0</v>
@@ -2652,14 +2734,1425 @@
       </c>
       <c r="N42" s="1"/>
       <c r="O42" s="1" t="n">
+        <v>18.0</v>
+      </c>
+      <c r="P42" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q42" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B43" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>Adama DABO</t>
+        </is>
+      </c>
+      <c r="H43" s="1"/>
+      <c r="I43" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 200gx10</t>
+        </is>
+      </c>
+      <c r="J43" s="1" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>12000.0</v>
+      </c>
+      <c r="L43" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M43" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N43" s="1"/>
+      <c r="O43" s="1" t="n">
+        <v>19.0</v>
+      </c>
+      <c r="P43" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q43" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>Saly THIOUNE (T2)</t>
+        </is>
+      </c>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>11000.0</v>
+      </c>
+      <c r="L44" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M44" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N44" s="1"/>
+      <c r="O44" s="1" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="P44" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q44" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>Sokhna (T2)</t>
+        </is>
+      </c>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J45" s="1" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>22000.0</v>
+      </c>
+      <c r="L45" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M45" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N45" s="1"/>
+      <c r="O45" s="1" t="n">
+        <v>21.0</v>
+      </c>
+      <c r="P45" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q45" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>Sokhna (T2)</t>
+        </is>
+      </c>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 200gx10</t>
+        </is>
+      </c>
+      <c r="J46" s="1" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>6000.0</v>
+      </c>
+      <c r="L46" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M46" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N46" s="1"/>
+      <c r="O46" s="1" t="n">
+        <v>22.0</v>
+      </c>
+      <c r="P46" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q46" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B47" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>Nogueye THIAME (T2)</t>
+        </is>
+      </c>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J47" s="1" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="K47" s="1" t="n">
+        <v>110000.0</v>
+      </c>
+      <c r="L47" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M47" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N47" s="1"/>
+      <c r="O47" s="1" t="n">
+        <v>23.0</v>
+      </c>
+      <c r="P47" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q47" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B48" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>Coumba Touré (T2)</t>
+        </is>
+      </c>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J48" s="1" t="n">
+        <v>11.0</v>
+      </c>
+      <c r="K48" s="1" t="n">
+        <v>121000.0</v>
+      </c>
+      <c r="L48" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M48" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N48" s="1"/>
+      <c r="O48" s="1" t="n">
+        <v>24.0</v>
+      </c>
+      <c r="P48" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q48" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B49" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>Fama DIOUF</t>
+        </is>
+      </c>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J49" s="1" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>55000.0</v>
+      </c>
+      <c r="L49" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M49" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N49" s="1"/>
+      <c r="O49" s="1" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="P49" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q49" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B50" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>Mariama KANE</t>
+        </is>
+      </c>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J50" s="1" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>55000.0</v>
+      </c>
+      <c r="L50" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M50" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N50" s="1"/>
+      <c r="O50" s="1" t="n">
+        <v>26.0</v>
+      </c>
+      <c r="P50" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q50" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B51" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>Mariama KANE</t>
+        </is>
+      </c>
+      <c r="H51" s="1"/>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 200gx10</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>6000.0</v>
+      </c>
+      <c r="L51" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M51" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N51" s="1"/>
+      <c r="O51" s="1" t="n">
+        <v>27.0</v>
+      </c>
+      <c r="P51" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q51" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B52" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>Fallou SOLY (T2)</t>
+        </is>
+      </c>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J52" s="1" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>165000.0</v>
+      </c>
+      <c r="L52" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M52" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1" t="n">
+        <v>28.0</v>
+      </c>
+      <c r="P52" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q52" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B53" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>Fallou SOLY (T2)</t>
+        </is>
+      </c>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>Cafe au Lait 3-en-1</t>
+        </is>
+      </c>
+      <c r="J53" s="1" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>4500.0</v>
+      </c>
+      <c r="L53" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M53" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N53" s="1"/>
+      <c r="O53" s="1" t="n">
+        <v>29.0</v>
+      </c>
+      <c r="P53" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q53" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B54" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>Vente</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>Mariama BA</t>
+        </is>
+      </c>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J54" s="1" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>110000.0</v>
+      </c>
+      <c r="L54" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M54" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N54" s="1"/>
+      <c r="O54" s="1" t="n">
+        <v>30.0</v>
+      </c>
+      <c r="P54" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q54" s="1" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B55" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1" t="inlineStr">
+        <is>
+          <t>Cafe au Lait 3-en-1</t>
+        </is>
+      </c>
+      <c r="J55" s="1" t="n">
+        <v>99.0</v>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>445500.0</v>
+      </c>
+      <c r="L55" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M55" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N55" s="1"/>
+      <c r="O55" s="1" t="n">
+        <v>31.0</v>
+      </c>
+      <c r="P55" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q55" s="1"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D56" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1" t="inlineStr">
+        <is>
+          <t>Chocolat 3-en-1 30x120 pcs</t>
+        </is>
+      </c>
+      <c r="J56" s="1" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>1100000.0</v>
+      </c>
+      <c r="L56" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M56" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N56" s="1"/>
+      <c r="O56" s="1" t="n">
+        <v>32.0</v>
+      </c>
+      <c r="P56" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q56" s="1"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B57" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+      <c r="I57" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 200gx10</t>
+        </is>
+      </c>
+      <c r="J57" s="1" t="n">
+        <v>134.0</v>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>804000.0</v>
+      </c>
+      <c r="L57" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M57" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N57" s="1"/>
+      <c r="O57" s="1" t="n">
+        <v>33.0</v>
+      </c>
+      <c r="P57" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q57" s="1"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D58" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1" t="inlineStr">
+        <is>
+          <t>Cowmilk 5kg</t>
+        </is>
+      </c>
+      <c r="J58" s="1" t="n">
+        <v>16.0</v>
+      </c>
+      <c r="K58" s="1" t="n">
+        <v>176000.0</v>
+      </c>
+      <c r="L58" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M58" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N58" s="1"/>
+      <c r="O58" s="1" t="n">
+        <v>34.0</v>
+      </c>
+      <c r="P58" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q58" s="1"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B59" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+      <c r="I59" s="1" t="inlineStr">
+        <is>
+          <t>Jus Lido</t>
+        </is>
+      </c>
+      <c r="J59" s="1" t="n">
+        <v>200.0</v>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>2200000.0</v>
+      </c>
+      <c r="L59" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M59" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N59" s="1"/>
+      <c r="O59" s="1" t="n">
+        <v>35.0</v>
+      </c>
+      <c r="P59" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q59" s="1"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B60" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D60" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F60" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Junior BLE cereal 230g x 12 sachet</t>
+        </is>
+      </c>
+      <c r="J60" s="1" t="n">
+        <v>24.416666</v>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>219750.0</v>
+      </c>
+      <c r="L60" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M60" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N60" s="1"/>
+      <c r="O60" s="1" t="n">
+        <v>36.0</v>
+      </c>
+      <c r="P60" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q60" s="1"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B61" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
+      <c r="I61" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Junior BLE cereal 50g x 10 x 8 sachet</t>
+        </is>
+      </c>
+      <c r="J61" s="1" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>375000.0</v>
+      </c>
+      <c r="L61" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M61" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N61" s="1"/>
+      <c r="O61" s="1" t="n">
+        <v>37.0</v>
+      </c>
+      <c r="P61" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q61" s="1"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+      <c r="I62" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Junior mais cereal 230g x 12 sachet</t>
+        </is>
+      </c>
+      <c r="J62" s="1" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>225000.0</v>
+      </c>
+      <c r="L62" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M62" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N62" s="1"/>
+      <c r="O62" s="1" t="n">
+        <v>38.0</v>
+      </c>
+      <c r="P62" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q62" s="1"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B63" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+      <c r="I63" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Junior mais cereal 50g x 10 x 8 sachet</t>
+        </is>
+      </c>
+      <c r="J63" s="1" t="n">
+        <v>25.0</v>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>375000.0</v>
+      </c>
+      <c r="L63" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M63" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N63" s="1"/>
+      <c r="O63" s="1" t="n">
+        <v>39.0</v>
+      </c>
+      <c r="P63" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q63" s="1"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D64" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F64" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+      <c r="I64" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac Thé 7g</t>
+        </is>
+      </c>
+      <c r="J64" s="1" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>1150000.0</v>
+      </c>
+      <c r="L64" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M64" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N64" s="1"/>
+      <c r="O64" s="1" t="n">
+        <v>40.0</v>
+      </c>
+      <c r="P64" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q64" s="1"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46221.0</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>TATA 1</t>
+        </is>
+      </c>
+      <c r="D65" s="1" t="inlineStr">
+        <is>
+          <t>DJIBRIL DIOP</t>
+        </is>
+      </c>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>Stock Descente</t>
+        </is>
+      </c>
+      <c r="F65" s="1" t="inlineStr">
+        <is>
+          <t>TOUBA</t>
+        </is>
+      </c>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1"/>
+      <c r="I65" s="1" t="inlineStr">
+        <is>
+          <t>Kamlac évaporé 48x160g</t>
+        </is>
+      </c>
+      <c r="J65" s="1" t="n">
+        <v>599.0</v>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>6289500.0</v>
+      </c>
+      <c r="L65" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M65" s="1" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N65" s="1"/>
+      <c r="O65" s="1" t="n">
         <v>41.0</v>
       </c>
-      <c r="P42" s="1" t="inlineStr">
-        <is>
-          <t>S29</t>
-        </is>
-      </c>
-      <c r="Q42" s="1"/>
+      <c r="P65" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="Q65" s="1"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Rapport du 26 Juillet 2026
</commit_message>
<xml_diff>
--- a/Donnees_Promoteurs.xlsx
+++ b/Donnees_Promoteurs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4F2A645-6CC9-4F20-9056-BE008CDB5822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C671998-B105-4B76-97C6-A88CF1CB72B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2372" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2368" uniqueCount="51">
   <si>
     <t>Date</t>
   </si>
@@ -2221,9 +2221,6 @@
         <v>20</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H34" s="1" t="s">
         <v>42</v>
       </c>
       <c r="I34" s="1" t="s">
@@ -2272,9 +2269,6 @@
         <v>20</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H35" s="1" t="s">
         <v>42</v>
       </c>
       <c r="I35" s="1" t="s">
@@ -2323,9 +2317,6 @@
         <v>20</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H36" s="1" t="s">
         <v>43</v>
       </c>
       <c r="I36" s="1" t="s">
@@ -2374,9 +2365,6 @@
         <v>20</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H37" s="1" t="s">
         <v>43</v>
       </c>
       <c r="I37" s="1" t="s">

</xml_diff>

<commit_message>
Rapport du 28 Juillet 2026
</commit_message>
<xml_diff>
--- a/Donnees_Promoteurs.xlsx
+++ b/Donnees_Promoteurs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73777F8-7FC5-4A3D-97F8-A96B1253A086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F856A35-E982-46E5-8512-87313FA2CCBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3111" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3113" uniqueCount="51">
   <si>
     <t>Date</t>
   </si>
@@ -1437,6 +1437,9 @@
         <v>20</v>
       </c>
       <c r="G18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>38</v>
       </c>
       <c r="I18" s="1" t="s">
@@ -1485,6 +1488,9 @@
         <v>20</v>
       </c>
       <c r="G19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>39</v>
       </c>
       <c r="I19" s="1" t="s">
@@ -1517,7 +1523,9 @@
       <c r="A20" s="2">
         <v>46232</v>
       </c>
-      <c r="B20" s="1"/>
+      <c r="B20" s="1">
+        <v>0</v>
+      </c>
       <c r="C20" s="1" t="s">
         <v>17</v>
       </c>
@@ -1536,10 +1544,10 @@
         <v>33</v>
       </c>
       <c r="J20" s="1">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K20" s="1">
-        <v>275000</v>
+        <v>264000</v>
       </c>
       <c r="L20" s="1">
         <v>0</v>
@@ -1560,7 +1568,9 @@
       <c r="A21" s="2">
         <v>46232</v>
       </c>
-      <c r="B21" s="1"/>
+      <c r="B21" s="1">
+        <v>0</v>
+      </c>
       <c r="C21" s="1" t="s">
         <v>17</v>
       </c>
@@ -1582,7 +1592,7 @@
         <v>1000</v>
       </c>
       <c r="K21" s="1">
-        <v>9000000</v>
+        <v>8500000</v>
       </c>
       <c r="L21" s="1">
         <v>0</v>

</xml_diff>

<commit_message>
Rapport du 10 Aout 2026
</commit_message>
<xml_diff>
--- a/Donnees_Promoteurs.xlsx
+++ b/Donnees_Promoteurs.xlsx
@@ -2317,7 +2317,7 @@
         <v>35.0</v>
       </c>
       <c r="K38" s="1" t="n">
-        <v>358750.0</v>
+        <v>393750.0</v>
       </c>
       <c r="L38" s="1" t="n">
         <v>0.0</v>
@@ -4460,7 +4460,7 @@
         <v>1.0</v>
       </c>
       <c r="K77" s="1" t="n">
-        <v>10250.0</v>
+        <v>11250.0</v>
       </c>
       <c r="L77" s="1" t="n">
         <v>0.0</v>
@@ -4915,7 +4915,7 @@
         <v>1.0</v>
       </c>
       <c r="K84" s="1" t="n">
-        <v>10250.0</v>
+        <v>11250.0</v>
       </c>
       <c r="L84" s="1" t="n">
         <v>0.0</v>
@@ -5870,7 +5870,7 @@
         <v>35.0</v>
       </c>
       <c r="K99" s="1" t="n">
-        <v>358750.0</v>
+        <v>393750.0</v>
       </c>
       <c r="L99" s="1" t="n">
         <v>0.0</v>
@@ -6241,7 +6241,7 @@
         <v>20.0</v>
       </c>
       <c r="K106" s="1" t="n">
-        <v>210000.0</v>
+        <v>180000.0</v>
       </c>
       <c r="L106" s="1" t="n">
         <v>0.0</v>
@@ -7068,7 +7068,7 @@
         <v>3.0</v>
       </c>
       <c r="K121" s="1" t="n">
-        <v>30750.0</v>
+        <v>33750.0</v>
       </c>
       <c r="L121" s="1" t="n">
         <v>0.0</v>
@@ -7198,7 +7198,7 @@
         <v>1.0</v>
       </c>
       <c r="K123" s="1" t="n">
-        <v>10250.0</v>
+        <v>11250.0</v>
       </c>
       <c r="L123" s="1" t="n">
         <v>0.0</v>

</xml_diff>